<commit_message>
Publish 2026-10-23 03:55 UTC (src d471594-dirty)
</commit_message>
<xml_diff>
--- a/Data/Wyndor_Uncertainty.xlsx
+++ b/Data/Wyndor_Uncertainty.xlsx
@@ -251,7 +251,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wyndor, robust counterpart: every parameter at its worst value (Hillier and Lieberman 11e, pp. 266-267)</t>
+          <t xml:space="preserve">Wyndor, robust counterpart: every parameter at its worst value</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wyndor with chance constraints: hours are normal (Hillier and Lieberman 11e, pp. 269-271)</t>
+          <t xml:space="preserve">Wyndor with chance constraints: hours are normal</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wyndor with recourse: doors now, windows after the rumor resolves (Hillier and Lieberman 11e, pp. 272-275)</t>
+          <t xml:space="preserve">Wyndor with recourse: doors now, windows after the rumor resolves</t>
         </is>
       </c>
     </row>

</xml_diff>